<commit_message>
Add chat session and update session/timing data
Update evaluation spreadsheet, add a new chat session JSON, and append timing metadata. Modified Data/evaluation/query_responses.xlsx (binary update), added Data/user_sessions/ChatSessions/chat_session_20260411_182759.json containing a user question and assistant response about importing qualitative data, updated Data/user_sessions/session_metadata.json to register the new session (and minor punctuation tweak to an existing title), and appended three entries to Data/user_sessions/timed_responses.json to record response times for the new session. These changes record a new user interaction and its timing for evaluation purposes.
</commit_message>
<xml_diff>
--- a/Data/evaluation/query_responses.xlsx
+++ b/Data/evaluation/query_responses.xlsx
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C338"/>
+  <dimension ref="A1:C339"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="96" customWidth="1" min="1" max="1"/>
@@ -434,17 +422,17 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Question</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Model Name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Response</t>
         </is>
@@ -6342,6 +6330,25 @@
         </is>
       </c>
     </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>What are the steps taken to import qualitative data?</t>
+        </is>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>llama3.2:latest</t>
+        </is>
+      </c>
+      <c r="C339" t="inlineStr">
+        <is>
+          <t>Option 1: SelectTrackSettings from the Edit menu, then select Import from File, browse to the .txt file, select it and Open, and click OK to exit Qualitative Track Information.
+Option 2: SelectTrackSettings from the Edit menu, then select Details on the qualitative track, select Import from File, browse to the .txt file, select it and Open, and click OK to exit Qualitative Track Information.
+Option 3: SelectTrackSettings from the Edit menu, then select Export to File or Export to Clipboard, select the desired export option, browse to the location or external application, enter a file name if exporting to file, and paste the contents of the clipboard if exporting to clipboard.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Store and serve raw AI responses; CSS cleanup
Stop post-processing AI output and send/store raw text: remove markdown-to-HTML formatting in question_handler.py and offline-app.py, update SSE endpoints in app/routes/api.py and offline-app.py to stream raw responses, and update ollama prompt to require plain-text, one-option-per-line output. Add a new chat session (Data/user_sessions/ChatSessions/chat_session_20260415_173914.json) and register it in session_metadata.json and timed_responses.json. Large CSS cleanup and enhancements in static/css/index.css and static/css/output.css (formatting fixes, spacing/consistency changes, new response-option styles and UI tweaks). Also update templates/chathistory.html and Data/evaluation/query_responses.xlsx (binary diff).
</commit_message>
<xml_diff>
--- a/Data/evaluation/query_responses.xlsx
+++ b/Data/evaluation/query_responses.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C339"/>
+  <dimension ref="A1:C340"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="96" customWidth="1" min="1" max="1"/>
@@ -6349,6 +6349,25 @@
         </is>
       </c>
     </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>What are the steps taken to import qualitative data?</t>
+        </is>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>llama3.2:latest</t>
+        </is>
+      </c>
+      <c r="C340" t="inlineStr">
+        <is>
+          <t>Option 1: SelectTrackSettings, then selectImport from File, browse to the .txt file, select it and Open, and click OK to exit Qualitative Track Information.
+Option 2: SelectTrackSettings, then select the qualitative track, selectDetails, selectImport from File, browse to the .txt file, select it and Open, and click OK to exit Qualitative Track Information.
+Option 3: SelectTrackSettings, then select the qualitative track you wish to export data from, selectDetails, Export to File, save the file in a location of your choice.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add GIS-limits chat session and update metadata
Add a new chat session (data/user_sessions/ChatSessions/chat_session_20260613_112913_58d515ab.json) recording a user question about GIS field limits and the assistant reply. Update Data/user_sessions/session_metadata.json to include the new session title mapping, and append the corresponding timed response entry to Data/user_sessions/timed_responses.json (response_time 60.08, timestamp 2026-06-13T10:30:13.595Z). Also include a binary update to Data/evaluation/query_responses.xlsx.
</commit_message>
<xml_diff>
--- a/Data/evaluation/query_responses.xlsx
+++ b/Data/evaluation/query_responses.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C340"/>
+  <dimension ref="A1:C341"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="96" customWidth="1" min="1" max="1"/>
@@ -6368,6 +6368,25 @@
         </is>
       </c>
     </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>What are the limits of GIS fields in GEO?</t>
+        </is>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>llama3.2:latest</t>
+        </is>
+      </c>
+      <c r="C341" t="inlineStr">
+        <is>
+          <t>Option 1: No specific limit is mentioned for GIS fields in the provided documents.
+Option 2: The provided documents do not mention any limits for GIS fields.
+Option 3: There is no information available on limits for GIS fields within GEO.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Improve chat UI/stability and streaming handling
Add two new chat session exports and update session metadata/timed responses; update binary query_responses.xlsx. Apply layout/CSS fixes to chathistory and chathistory_v2 to stabilize full-height layout and keep composer/input out of the streamed answer area. Harden streaming logic: use encodeURIComponent for EventSource URLs, ignore transient status messages, detect stream completion tokens, add an idle finalize timeout, and ensure smooth auto-scroll behavior. Improve UX and safety by escaping user content when rendering, clearing initial placeholders when loading new chats, adding response-time display, and preventing duplicate feedback containers. Small UI tweaks (buttons/text) and assorted DOM/flow fixes to ensure consistent streaming, finalization, and timing storage to /store-response-time.
</commit_message>
<xml_diff>
--- a/Data/evaluation/query_responses.xlsx
+++ b/Data/evaluation/query_responses.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C341"/>
+  <dimension ref="A1:C343"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="96" customWidth="1" min="1" max="1"/>
@@ -6387,6 +6387,44 @@
         </is>
       </c>
     </row>
+    <row r="342">
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>How do I import qualitative data into GEO?</t>
+        </is>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>llama3.2:latest</t>
+        </is>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>Option 1: Export to File; select Export to File, browse to a location, enter a file name, and select Save.
+Option 2: Export to Clipboard; select Export to Clipboard, open an external application (i.e. Excel), paste the contents of your clipboard.
+Option 3: Import from File; select Import from File, browse to the .txt file, select it, and Open.</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>What are the limits of GIS fields in GEO?</t>
+        </is>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>llama3.2:latest</t>
+        </is>
+      </c>
+      <c r="C343" t="inlineStr">
+        <is>
+          <t>Option 1: No specific limit is mentioned for GIS fields in the provided documents.
+Option 2: The provided documents do not mention any limits for GIS fields.
+Option 3: There is no information available on limits for GIS fields within GEO.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>